<commit_message>
Sync model-ledger data written by the live daily pipeline mid-session
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/model_ledgers/mlb-spread-measured-edge.xlsx
+++ b/data/model_ledgers/mlb-spread-measured-edge.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Predictions" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Predictions'!$A$1:$AJ$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Predictions'!$A$1:$AJ$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ69"/>
+  <dimension ref="A1:AJ70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -9456,8 +9456,126 @@
       <c r="AI69" s="2" t="inlineStr"/>
       <c r="AJ69" s="2" t="inlineStr"/>
     </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>85eefd84a9614a40</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>mlb-spread-measured-edge</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>measured-edge-margin-v2</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>8360b122264b796b0fb193095cfe4506c7e064e5f3f8c0a659aec41efd08dd25</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>measured-edge-paired-v1</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>v3</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>401816372</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="inlineStr">
+        <is>
+          <t>spread</t>
+        </is>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>away</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="inlineStr">
+        <is>
+          <t>0.632943</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr"/>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>0.042131</t>
+        </is>
+      </c>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>0.559471</t>
+        </is>
+      </c>
+      <c r="P70" s="2" t="inlineStr">
+        <is>
+          <t>0.557214</t>
+        </is>
+      </c>
+      <c r="Q70" s="2" t="inlineStr">
+        <is>
+          <t>0.073472</t>
+        </is>
+      </c>
+      <c r="R70" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02T15:47:52.139141Z</t>
+        </is>
+      </c>
+      <c r="S70" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-02T23:20Z</t>
+        </is>
+      </c>
+      <c r="T70" s="2" t="inlineStr"/>
+      <c r="U70" s="2" t="inlineStr"/>
+      <c r="V70" s="2" t="inlineStr"/>
+      <c r="W70" s="2" t="inlineStr">
+        <is>
+          <t>migrated_from=data/flat_picks.xlsx;original_pick_id=85eefd84a9614a40;original_record_type=QUALIFIED_SHADOW_CALL</t>
+        </is>
+      </c>
+      <c r="X70" s="2" t="inlineStr">
+        <is>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="Y70" s="2" t="inlineStr"/>
+      <c r="Z70" s="2" t="inlineStr"/>
+      <c r="AA70" s="2" t="inlineStr"/>
+      <c r="AB70" s="2" t="inlineStr"/>
+      <c r="AC70" s="2" t="inlineStr"/>
+      <c r="AD70" s="2" t="inlineStr"/>
+      <c r="AE70" s="2" t="inlineStr"/>
+      <c r="AF70" s="2" t="inlineStr"/>
+      <c r="AG70" s="2" t="inlineStr"/>
+      <c r="AH70" s="2" t="inlineStr"/>
+      <c r="AI70" s="2" t="inlineStr"/>
+      <c r="AJ70" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AJ69"/>
+  <autoFilter ref="A1:AJ70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>